<commit_message>
Familles : reprise de l'axe officiel, lu dans le code de la fiche
Les familles que j'avais écrites étaient inventées, et elles contredisaient déjà
les codes : BAT-EQ-127 était rangé dans « Éclairage » alors que son segment dit EQ.

Le champ `famille` disparaît de la table. La famille est le deuxième segment du
code officiel ; lib/familles.ts ne fait que lui donner un libellé et dire dans
quels secteurs il existe. Une fiche ne peut plus être mal rangée, son rangement
vient de son propre code.

Deux contrôles au build, éprouvés en falsifiant un code :
- segment inconnu (IND-ZZ-110) : arrêt ;
- segment réel mais impossible dans ce secteur (IND-TH-110) : arrêt. C'est à quoi
  ressemble une ligne mal recopiée du catalogue officiel — elle se compile et
  s'affiche sans broncher.

Les sections d'un hub sont déduites des codes présents, plus d'une liste déclarée :
un hub ne peut plus afficher une section vide ni oublier une famille dont il a des
fiches.
</commit_message>
<xml_diff>
--- a/data/fiches_cee.xlsx
+++ b/data/fiches_cee.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alek/Documents/Projets/Ultra Energie/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47754ABC-9CFA-8F49-9EEE-7ECC7A4D571A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A54EA54F-8001-F04E-BBFB-7644543E60FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{BA93B3AD-2B97-4542-BD80-901C18E74C66}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$C$219</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$C$217</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="233">
   <si>
     <t>secteur</t>
   </si>
@@ -738,12 +738,6 @@
   </si>
   <si>
     <t>TRA-SE-117</t>
-  </si>
-  <si>
-    <t>BAR-TH-159</t>
-  </si>
-  <si>
-    <t>TRA-EQ-132</t>
   </si>
 </sst>
 </file>
@@ -1129,7 +1123,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AACFCB85-DFF1-ED41-A31D-2937C9C48D6B}">
-  <dimension ref="A1:C219"/>
+  <dimension ref="A1:C217"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="27" customWidth="1"/>
@@ -1891,7 +1885,7 @@
         <v>23</v>
       </c>
       <c r="C69" t="s">
-        <v>233</v>
+        <v>81</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
@@ -1902,7 +1896,7 @@
         <v>23</v>
       </c>
       <c r="C70" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -1913,7 +1907,7 @@
         <v>23</v>
       </c>
       <c r="C71" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
@@ -1924,7 +1918,7 @@
         <v>23</v>
       </c>
       <c r="C72" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
@@ -1935,7 +1929,7 @@
         <v>23</v>
       </c>
       <c r="C73" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
@@ -1946,7 +1940,7 @@
         <v>23</v>
       </c>
       <c r="C74" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
@@ -1957,7 +1951,7 @@
         <v>23</v>
       </c>
       <c r="C75" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -1968,7 +1962,7 @@
         <v>23</v>
       </c>
       <c r="C76" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
@@ -1979,7 +1973,7 @@
         <v>23</v>
       </c>
       <c r="C77" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
@@ -1990,7 +1984,7 @@
         <v>23</v>
       </c>
       <c r="C78" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
@@ -2001,7 +1995,7 @@
         <v>23</v>
       </c>
       <c r="C79" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
@@ -2012,7 +2006,7 @@
         <v>23</v>
       </c>
       <c r="C80" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
@@ -2023,7 +2017,7 @@
         <v>23</v>
       </c>
       <c r="C81" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
@@ -2034,7 +2028,7 @@
         <v>23</v>
       </c>
       <c r="C82" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
@@ -2045,7 +2039,7 @@
         <v>23</v>
       </c>
       <c r="C83" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
@@ -2056,18 +2050,18 @@
         <v>23</v>
       </c>
       <c r="C84" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B85" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="C85" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
@@ -2078,7 +2072,7 @@
         <v>41</v>
       </c>
       <c r="C86" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
@@ -2089,7 +2083,7 @@
         <v>41</v>
       </c>
       <c r="C87" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
@@ -2100,7 +2094,7 @@
         <v>41</v>
       </c>
       <c r="C88" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
@@ -2111,7 +2105,7 @@
         <v>41</v>
       </c>
       <c r="C89" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
@@ -2122,7 +2116,7 @@
         <v>41</v>
       </c>
       <c r="C90" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
@@ -2133,7 +2127,7 @@
         <v>41</v>
       </c>
       <c r="C91" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
@@ -2144,7 +2138,7 @@
         <v>41</v>
       </c>
       <c r="C92" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
@@ -2155,7 +2149,7 @@
         <v>41</v>
       </c>
       <c r="C93" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
@@ -2166,7 +2160,7 @@
         <v>41</v>
       </c>
       <c r="C94" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
@@ -2177,7 +2171,7 @@
         <v>41</v>
       </c>
       <c r="C95" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
@@ -2188,7 +2182,7 @@
         <v>41</v>
       </c>
       <c r="C96" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
@@ -2196,10 +2190,10 @@
         <v>3</v>
       </c>
       <c r="B97" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="C97" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
@@ -2210,7 +2204,7 @@
         <v>8</v>
       </c>
       <c r="C98" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
@@ -2221,7 +2215,7 @@
         <v>8</v>
       </c>
       <c r="C99" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
@@ -2232,7 +2226,7 @@
         <v>8</v>
       </c>
       <c r="C100" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
@@ -2243,7 +2237,7 @@
         <v>8</v>
       </c>
       <c r="C101" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
@@ -2254,7 +2248,7 @@
         <v>8</v>
       </c>
       <c r="C102" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
@@ -2265,7 +2259,7 @@
         <v>8</v>
       </c>
       <c r="C103" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
@@ -2276,7 +2270,7 @@
         <v>8</v>
       </c>
       <c r="C104" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
@@ -2287,7 +2281,7 @@
         <v>8</v>
       </c>
       <c r="C105" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
@@ -2295,10 +2289,10 @@
         <v>3</v>
       </c>
       <c r="B106" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C106" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
@@ -2309,7 +2303,7 @@
         <v>21</v>
       </c>
       <c r="C107" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
@@ -2320,7 +2314,7 @@
         <v>21</v>
       </c>
       <c r="C108" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.2">
@@ -2328,10 +2322,10 @@
         <v>3</v>
       </c>
       <c r="B109" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C109" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
@@ -2342,7 +2336,7 @@
         <v>23</v>
       </c>
       <c r="C110" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.2">
@@ -2353,7 +2347,7 @@
         <v>23</v>
       </c>
       <c r="C111" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
@@ -2364,7 +2358,7 @@
         <v>23</v>
       </c>
       <c r="C112" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
@@ -2375,7 +2369,7 @@
         <v>23</v>
       </c>
       <c r="C113" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
@@ -2386,7 +2380,7 @@
         <v>23</v>
       </c>
       <c r="C114" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
@@ -2397,7 +2391,7 @@
         <v>23</v>
       </c>
       <c r="C115" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
@@ -2408,7 +2402,7 @@
         <v>23</v>
       </c>
       <c r="C116" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
@@ -2419,7 +2413,7 @@
         <v>23</v>
       </c>
       <c r="C117" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
@@ -2430,7 +2424,7 @@
         <v>23</v>
       </c>
       <c r="C118" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
@@ -2441,7 +2435,7 @@
         <v>23</v>
       </c>
       <c r="C119" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
@@ -2452,7 +2446,7 @@
         <v>23</v>
       </c>
       <c r="C120" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
@@ -2463,7 +2457,7 @@
         <v>23</v>
       </c>
       <c r="C121" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
@@ -2474,7 +2468,7 @@
         <v>23</v>
       </c>
       <c r="C122" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
@@ -2485,7 +2479,7 @@
         <v>23</v>
       </c>
       <c r="C123" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
@@ -2496,7 +2490,7 @@
         <v>23</v>
       </c>
       <c r="C124" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
@@ -2507,7 +2501,7 @@
         <v>23</v>
       </c>
       <c r="C125" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
@@ -2518,7 +2512,7 @@
         <v>23</v>
       </c>
       <c r="C126" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
@@ -2529,7 +2523,7 @@
         <v>23</v>
       </c>
       <c r="C127" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.2">
@@ -2540,7 +2534,7 @@
         <v>23</v>
       </c>
       <c r="C128" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
@@ -2551,7 +2545,7 @@
         <v>23</v>
       </c>
       <c r="C129" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
@@ -2562,7 +2556,7 @@
         <v>23</v>
       </c>
       <c r="C130" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
@@ -2573,7 +2567,7 @@
         <v>23</v>
       </c>
       <c r="C131" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
@@ -2584,7 +2578,7 @@
         <v>23</v>
       </c>
       <c r="C132" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.2">
@@ -2595,7 +2589,7 @@
         <v>23</v>
       </c>
       <c r="C133" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
@@ -2606,7 +2600,7 @@
         <v>23</v>
       </c>
       <c r="C134" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
@@ -2617,7 +2611,7 @@
         <v>23</v>
       </c>
       <c r="C135" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
@@ -2628,7 +2622,7 @@
         <v>23</v>
       </c>
       <c r="C136" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.2">
@@ -2639,7 +2633,7 @@
         <v>23</v>
       </c>
       <c r="C137" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.2">
@@ -2650,18 +2644,18 @@
         <v>23</v>
       </c>
       <c r="C138" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B139" t="s">
-        <v>23</v>
+        <v>151</v>
       </c>
       <c r="C139" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
@@ -2672,7 +2666,7 @@
         <v>151</v>
       </c>
       <c r="C140" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.2">
@@ -2683,7 +2677,7 @@
         <v>151</v>
       </c>
       <c r="C141" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.2">
@@ -2694,7 +2688,7 @@
         <v>151</v>
       </c>
       <c r="C142" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.2">
@@ -2702,10 +2696,10 @@
         <v>4</v>
       </c>
       <c r="B143" t="s">
-        <v>151</v>
+        <v>41</v>
       </c>
       <c r="C143" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.2">
@@ -2716,7 +2710,7 @@
         <v>41</v>
       </c>
       <c r="C144" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.2">
@@ -2724,10 +2718,10 @@
         <v>4</v>
       </c>
       <c r="B145" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C145" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.2">
@@ -2738,7 +2732,7 @@
         <v>36</v>
       </c>
       <c r="C146" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.2">
@@ -2749,7 +2743,7 @@
         <v>36</v>
       </c>
       <c r="C147" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.2">
@@ -2760,7 +2754,7 @@
         <v>36</v>
       </c>
       <c r="C148" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.2">
@@ -2771,7 +2765,7 @@
         <v>36</v>
       </c>
       <c r="C149" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.2">
@@ -2782,7 +2776,7 @@
         <v>36</v>
       </c>
       <c r="C150" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.2">
@@ -2793,7 +2787,7 @@
         <v>36</v>
       </c>
       <c r="C151" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.2">
@@ -2804,7 +2798,7 @@
         <v>36</v>
       </c>
       <c r="C152" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.2">
@@ -2815,7 +2809,7 @@
         <v>36</v>
       </c>
       <c r="C153" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
@@ -2826,7 +2820,7 @@
         <v>36</v>
       </c>
       <c r="C154" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
@@ -2837,7 +2831,7 @@
         <v>36</v>
       </c>
       <c r="C155" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.2">
@@ -2848,7 +2842,7 @@
         <v>36</v>
       </c>
       <c r="C156" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.2">
@@ -2859,7 +2853,7 @@
         <v>36</v>
       </c>
       <c r="C157" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
@@ -2870,7 +2864,7 @@
         <v>36</v>
       </c>
       <c r="C158" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
@@ -2881,7 +2875,7 @@
         <v>36</v>
       </c>
       <c r="C159" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.2">
@@ -2892,7 +2886,7 @@
         <v>36</v>
       </c>
       <c r="C160" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.2">
@@ -2903,7 +2897,7 @@
         <v>36</v>
       </c>
       <c r="C161" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.2">
@@ -2914,7 +2908,7 @@
         <v>36</v>
       </c>
       <c r="C162" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.2">
@@ -2925,7 +2919,7 @@
         <v>36</v>
       </c>
       <c r="C163" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.2">
@@ -2936,7 +2930,7 @@
         <v>36</v>
       </c>
       <c r="C164" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.2">
@@ -2947,7 +2941,7 @@
         <v>36</v>
       </c>
       <c r="C165" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.2">
@@ -2958,7 +2952,7 @@
         <v>36</v>
       </c>
       <c r="C166" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.2">
@@ -2969,7 +2963,7 @@
         <v>36</v>
       </c>
       <c r="C167" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.2">
@@ -2980,7 +2974,7 @@
         <v>36</v>
       </c>
       <c r="C168" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.2">
@@ -2991,18 +2985,18 @@
         <v>36</v>
       </c>
       <c r="C169" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B170" t="s">
-        <v>36</v>
+        <v>183</v>
       </c>
       <c r="C170" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.2">
@@ -3013,7 +3007,7 @@
         <v>183</v>
       </c>
       <c r="C171" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.2">
@@ -3024,7 +3018,7 @@
         <v>183</v>
       </c>
       <c r="C172" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.2">
@@ -3035,7 +3029,7 @@
         <v>183</v>
       </c>
       <c r="C173" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.2">
@@ -3046,7 +3040,7 @@
         <v>183</v>
       </c>
       <c r="C174" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.2">
@@ -3054,21 +3048,21 @@
         <v>5</v>
       </c>
       <c r="B175" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C175" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B176" t="s">
-        <v>189</v>
+        <v>8</v>
       </c>
       <c r="C176" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.2">
@@ -3079,7 +3073,7 @@
         <v>8</v>
       </c>
       <c r="C177" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.2">
@@ -3090,7 +3084,7 @@
         <v>8</v>
       </c>
       <c r="C178" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.2">
@@ -3101,7 +3095,7 @@
         <v>8</v>
       </c>
       <c r="C179" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.2">
@@ -3112,7 +3106,7 @@
         <v>8</v>
       </c>
       <c r="C180" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.2">
@@ -3123,7 +3117,7 @@
         <v>8</v>
       </c>
       <c r="C181" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.2">
@@ -3134,7 +3128,7 @@
         <v>8</v>
       </c>
       <c r="C182" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.2">
@@ -3145,7 +3139,7 @@
         <v>8</v>
       </c>
       <c r="C183" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.2">
@@ -3156,7 +3150,7 @@
         <v>8</v>
       </c>
       <c r="C184" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.2">
@@ -3167,7 +3161,7 @@
         <v>8</v>
       </c>
       <c r="C185" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.2">
@@ -3178,7 +3172,7 @@
         <v>8</v>
       </c>
       <c r="C186" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.2">
@@ -3189,7 +3183,7 @@
         <v>8</v>
       </c>
       <c r="C187" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.2">
@@ -3200,7 +3194,7 @@
         <v>8</v>
       </c>
       <c r="C188" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.2">
@@ -3211,7 +3205,7 @@
         <v>8</v>
       </c>
       <c r="C189" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.2">
@@ -3222,7 +3216,7 @@
         <v>8</v>
       </c>
       <c r="C190" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.2">
@@ -3233,7 +3227,7 @@
         <v>8</v>
       </c>
       <c r="C191" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.2">
@@ -3244,7 +3238,7 @@
         <v>8</v>
       </c>
       <c r="C192" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.2">
@@ -3255,7 +3249,7 @@
         <v>8</v>
       </c>
       <c r="C193" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.2">
@@ -3266,7 +3260,7 @@
         <v>8</v>
       </c>
       <c r="C194" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.2">
@@ -3277,7 +3271,7 @@
         <v>8</v>
       </c>
       <c r="C195" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.2">
@@ -3288,7 +3282,7 @@
         <v>8</v>
       </c>
       <c r="C196" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.2">
@@ -3299,7 +3293,7 @@
         <v>8</v>
       </c>
       <c r="C197" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.2">
@@ -3310,7 +3304,7 @@
         <v>8</v>
       </c>
       <c r="C198" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.2">
@@ -3321,7 +3315,7 @@
         <v>8</v>
       </c>
       <c r="C199" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.2">
@@ -3332,7 +3326,7 @@
         <v>8</v>
       </c>
       <c r="C200" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.2">
@@ -3343,7 +3337,7 @@
         <v>8</v>
       </c>
       <c r="C201" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.2">
@@ -3354,7 +3348,7 @@
         <v>8</v>
       </c>
       <c r="C202" t="s">
-        <v>217</v>
+        <v>203</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.2">
@@ -3365,7 +3359,7 @@
         <v>8</v>
       </c>
       <c r="C203" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.2">
@@ -3373,10 +3367,10 @@
         <v>6</v>
       </c>
       <c r="B204" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C204" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.2">
@@ -3384,10 +3378,10 @@
         <v>6</v>
       </c>
       <c r="B205" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C205" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.2">
@@ -3398,7 +3392,7 @@
         <v>21</v>
       </c>
       <c r="C206" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.2">
@@ -3409,7 +3403,7 @@
         <v>21</v>
       </c>
       <c r="C207" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.2">
@@ -3420,7 +3414,7 @@
         <v>21</v>
       </c>
       <c r="C208" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.2">
@@ -3431,7 +3425,7 @@
         <v>21</v>
       </c>
       <c r="C209" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.2">
@@ -3442,7 +3436,7 @@
         <v>21</v>
       </c>
       <c r="C210" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.2">
@@ -3453,7 +3447,7 @@
         <v>21</v>
       </c>
       <c r="C211" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.2">
@@ -3464,7 +3458,7 @@
         <v>21</v>
       </c>
       <c r="C212" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.2">
@@ -3475,7 +3469,7 @@
         <v>21</v>
       </c>
       <c r="C213" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.2">
@@ -3486,7 +3480,7 @@
         <v>21</v>
       </c>
       <c r="C214" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.2">
@@ -3497,7 +3491,7 @@
         <v>21</v>
       </c>
       <c r="C215" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.2">
@@ -3508,7 +3502,7 @@
         <v>21</v>
       </c>
       <c r="C216" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.2">
@@ -3519,33 +3513,11 @@
         <v>21</v>
       </c>
       <c r="C217" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A218" t="s">
-        <v>6</v>
-      </c>
-      <c r="B218" t="s">
-        <v>21</v>
-      </c>
-      <c r="C218" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A219" t="s">
-        <v>6</v>
-      </c>
-      <c r="B219" t="s">
-        <v>21</v>
-      </c>
-      <c r="C219" t="s">
         <v>232</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C219" xr:uid="{AACFCB85-DFF1-ED41-A31D-2937C9C48D6B}"/>
+  <autoFilter ref="A1:C217" xr:uid="{AACFCB85-DFF1-ED41-A31D-2937C9C48D6B}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>